<commit_message>
Updated CHN_grids_kan60 model - 2026-09-28 15:20
</commit_message>
<xml_diff>
--- a/VerveStacks_CHN_grids_kan60/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_CHN_grids_kan60/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHN_grids_kan60\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9103F4B-5595-4E5F-AD69-74CB989FEE40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD160850-C9F8-425B-A617-DBAFB89AE980}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1103" yWindow="1103" windowWidth="21600" windowHeight="12772" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3675" yWindow="3675" windowWidth="21600" windowHeight="11423" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap" sheetId="70" r:id="rId1"/>
@@ -6283,7 +6283,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A04AF3FE-3BBB-4CC7-AC99-43F77FEDF5EE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5958C3A6-E9F8-468F-A96C-FC31D9C97F79}">
   <dimension ref="B9:L460"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -43361,7 +43361,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7608B88-5D7C-490B-9FCA-301AAB83AA8A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9A7061A-71BF-459A-AE69-0C4602695E95}">
   <dimension ref="B9:H460"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CHN_grids_kan60 model - 2026-09-28 16:08
</commit_message>
<xml_diff>
--- a/VerveStacks_CHN_grids_kan60/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_CHN_grids_kan60/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHN_grids_kan60\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD160850-C9F8-425B-A617-DBAFB89AE980}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB9EA2EE-4BBC-485A-9D02-2F72CA826F98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3675" yWindow="3675" windowWidth="21600" windowHeight="11423" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6283,7 +6283,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5958C3A6-E9F8-468F-A96C-FC31D9C97F79}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAFB17CA-E100-4C5D-BF2C-18E88C389D90}">
   <dimension ref="B9:L460"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -43361,7 +43361,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9A7061A-71BF-459A-AE69-0C4602695E95}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDED0523-4F58-4BB8-8453-CB64EBF787B4}">
   <dimension ref="B9:H460"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CHN_grids_kan60 model - 2026-09-28 18:44
</commit_message>
<xml_diff>
--- a/VerveStacks_CHN_grids_kan60/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_CHN_grids_kan60/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHN_grids_kan60\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB9EA2EE-4BBC-485A-9D02-2F72CA826F98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BBC86B5-3873-4B13-988F-147F1FEFC67F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3675" yWindow="3675" windowWidth="21600" windowHeight="11423" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6283,7 +6283,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAFB17CA-E100-4C5D-BF2C-18E88C389D90}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C516D42F-3614-4BCE-AAA0-4CCEFF84AE64}">
   <dimension ref="B9:L460"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -43361,7 +43361,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDED0523-4F58-4BB8-8453-CB64EBF787B4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{810ECD66-0C68-4611-A80D-9BAA20FA45CA}">
   <dimension ref="B9:H460"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CHN_grids_kan60 model - 2026-09-28 19:10
</commit_message>
<xml_diff>
--- a/VerveStacks_CHN_grids_kan60/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_CHN_grids_kan60/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHN_grids_kan60\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BBC86B5-3873-4B13-988F-147F1FEFC67F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D462DDF2-E01F-48A4-A040-53ACB71B1F08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3675" yWindow="3675" windowWidth="21600" windowHeight="11423" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6283,7 +6283,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C516D42F-3614-4BCE-AAA0-4CCEFF84AE64}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B482869-6806-41B4-A4ED-1F80A8C62105}">
   <dimension ref="B9:L460"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -43361,7 +43361,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{810ECD66-0C68-4611-A80D-9BAA20FA45CA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97E0C9F0-81AC-4F6E-A041-873ED8FE8116}">
   <dimension ref="B9:H460"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>